<commit_message>
feat: add expression function library and aggregation support
- Expand derived-column expression evaluator with string, date, type-conversion,
  conditional, comparison, boolean, and numeric functions.
- Add optional grouping and aggregation sheets supporting count, count_distinct,
  sum, avg, min/max, first/last, and separator-based text join.
- Add aggregation tutorial and example workbook, expression-function tests, and
  refresh reference docs, examples, and changelog.

Co-Authored-By: GLM 5.1 <noreply@z.ai>
</commit_message>
<xml_diff>
--- a/examples/tutorial/01_single_sheet.xlsx
+++ b/examples/tutorial/01_single_sheet.xlsx
@@ -12,7 +12,9 @@
     <sheet name="关联关系" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="字段映射" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="过滤条件" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="填写说明" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="分组字段" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="聚合规则" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="填写说明" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'抽取计划'!$A$1:$C$2</definedName>
@@ -20,7 +22,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'关联关系'!$A$1:$G$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'字段映射'!$A$1:$G$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'过滤条件'!$A$1:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'填写说明'!$A$1:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'分组字段'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'聚合规则'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'填写说明'!$A$1:$B$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -871,7 +875,142 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>任务ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>源字段</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>目标字段</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>目标类型</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>分组顺序</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"integer,decimal,string,datetime"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>任务ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>源字段</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>聚合函数</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>目标字段</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>目标类型</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>分隔符</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>聚合顺序</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H1"/>
+  <dataValidations count="2">
+    <dataValidation sqref="C2:C5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"count,count_all,count_distinct,sum,avg,min,max,first,last,concat_agg"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"integer,decimal,string,datetime"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -946,48 +1085,60 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>支持 + - * / %、coalesce、abs、round，例如 coalesce(i.quantity, 0) * i.price</t>
+          <t>支持安全的数值、字符串、日期、条件函数；详见表达式参考</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>目标类型</t>
+          <t>分组聚合</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>从下拉框选择 integer、decimal、string 或 datetime，执行时会转换输出列类型</t>
+          <t>分组字段定义结果维度，聚合规则支持计数、求和、平均值、极值及文本合并；聚合任务不再执行字段映射</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>过滤条件</t>
+          <t>目标类型</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>同组内 AND，不同组之间 OR；IN 值用英文逗号分隔</t>
+          <t>从下拉框选择 integer、decimal、string 或 datetime，执行时会转换输出列类型</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>过滤条件</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>同组内 AND，不同组之间 OR；IN 值用英文逗号分隔</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>输出</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>执行 run 时分别指定输出格式（csv/jsonl/xlsx）和输出路径</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B9"/>
+  <autoFilter ref="A1:B10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>